<commit_message>
fixed csv file error
</commit_message>
<xml_diff>
--- a/AlphaFold/Benchmark set columns.xlsx
+++ b/AlphaFold/Benchmark set columns.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eigene Datein\Programmieren\Git\abrilka\bachelorthesis\AlphaFold\AF2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eigene Datein\Programmieren\Git\abrilka\bachelorthesis\AlphaFold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A15EFAF-CC79-4DD2-ADA0-735DE9560E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75DB871A-10BD-4A1F-A395-21247CB4DA14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D6D96FCB-1405-4904-B62B-E37067DD72C6}"/>
   </bookViews>
@@ -129,9 +129,6 @@
     <t>nearly all</t>
   </si>
   <si>
-    <t>Chain ID in the experimentally solved structure corrosponding to chain A in the AlphaFold prediction; Is always A for DMI. For DDI, the known_DDI prediction names contain the chain ID. Thats the reason why for some random_DDI without a known_DDI counterpart no chain ID is listed</t>
-  </si>
-  <si>
     <t>Chain ID in the experimentally solved structure corrosponding to chain A in the AlphaFold prediction</t>
   </si>
   <si>
@@ -487,6 +484,9 @@
   </si>
   <si>
     <t>Chain ID in the experimentally solved stucture, that corosponds to chain B in the AlphaFold prediction</t>
+  </si>
+  <si>
+    <t>Chain ID in the experimentally solved structure corrosponding to chain A in the AlphaFold prediction. Is always A for DMI. For DDI, the known_DDI prediction names contain the chain ID. Thats the reason why for some random_DDI without a known_DDI counterpart no chain ID is listed</t>
   </si>
 </sst>
 </file>
@@ -551,6 +551,20 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -567,20 +581,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-      </border>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -613,7 +613,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8B1E9C9E-7489-4911-A074-BC8F04372E9E}" name="Table2" displayName="Table2" ref="C7:G19" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8B1E9C9E-7489-4911-A074-BC8F04372E9E}" name="Table2" displayName="Table2" ref="C7:G19" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="C7:G19" xr:uid="{8B1E9C9E-7489-4911-A074-BC8F04372E9E}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F0CCD40F-B504-4D13-A0C3-E32515D436CD}" name="Column1"/>
@@ -956,12 +956,12 @@
   <sheetData>
     <row r="3" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="3:7" x14ac:dyDescent="0.25">
@@ -1079,7 +1079,7 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F14" t="s">
         <v>16</v>
@@ -1093,7 +1093,7 @@
         <v>24</v>
       </c>
       <c r="E15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
@@ -1113,7 +1113,7 @@
         <v>29</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>30</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" spans="3:7" x14ac:dyDescent="0.25">
@@ -1127,68 +1127,68 @@
         <v>29</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="3:7" ht="45" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F18" t="s">
         <v>29</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F20" t="s">
         <v>29</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" t="s">
+        <v>29</v>
+      </c>
+      <c r="G21" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="E21" t="s">
-        <v>61</v>
-      </c>
-      <c r="F21" t="s">
-        <v>29</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="22" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E22" t="s">
         <v>7</v>
@@ -1197,119 +1197,119 @@
         <v>16</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F23" t="s">
         <v>39</v>
       </c>
-      <c r="E23" t="s">
-        <v>7</v>
-      </c>
-      <c r="F23" t="s">
-        <v>40</v>
-      </c>
       <c r="G23" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="3:7" ht="30" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
+        <v>42</v>
+      </c>
+      <c r="E24" t="s">
+        <v>7</v>
+      </c>
+      <c r="F24" t="s">
         <v>43</v>
       </c>
-      <c r="E24" t="s">
-        <v>7</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="25" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E25" t="s">
         <v>7</v>
       </c>
       <c r="F25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G25" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="26" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
+        <v>49</v>
+      </c>
+      <c r="E26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F26" t="s">
+        <v>46</v>
+      </c>
+      <c r="G26" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="E26" t="s">
-        <v>7</v>
-      </c>
-      <c r="F26" t="s">
-        <v>47</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="27" spans="3:7" ht="30" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" t="s">
         <v>52</v>
       </c>
-      <c r="E27" t="s">
-        <v>7</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="28" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
+        <v>54</v>
+      </c>
+      <c r="E28" t="s">
+        <v>7</v>
+      </c>
+      <c r="F28" t="s">
         <v>55</v>
       </c>
-      <c r="E28" t="s">
-        <v>7</v>
-      </c>
-      <c r="F28" t="s">
-        <v>56</v>
-      </c>
       <c r="G28" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E29" t="s">
         <v>7</v>
       </c>
       <c r="F29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
+        <v>59</v>
+      </c>
+      <c r="E30" t="s">
         <v>60</v>
       </c>
-      <c r="E30" t="s">
-        <v>61</v>
-      </c>
       <c r="F30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="3:7" x14ac:dyDescent="0.25">
@@ -1317,16 +1317,16 @@
         <v>5</v>
       </c>
       <c r="D31" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F31" t="s">
         <v>16</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="32" spans="3:7" x14ac:dyDescent="0.25">
@@ -1334,16 +1334,16 @@
         <v>8</v>
       </c>
       <c r="D32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E32" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F32" t="s">
         <v>16</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="3:7" x14ac:dyDescent="0.25">
@@ -1351,16 +1351,16 @@
         <v>8</v>
       </c>
       <c r="D33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E33" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F33" t="s">
         <v>16</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="3:7" ht="30" x14ac:dyDescent="0.25">
@@ -1368,16 +1368,16 @@
         <v>8</v>
       </c>
       <c r="D34" t="s">
+        <v>67</v>
+      </c>
+      <c r="E34" t="s">
+        <v>78</v>
+      </c>
+      <c r="F34" t="s">
+        <v>16</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="E34" t="s">
-        <v>79</v>
-      </c>
-      <c r="F34" t="s">
-        <v>16</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="35" spans="3:7" x14ac:dyDescent="0.25">
@@ -1385,16 +1385,16 @@
         <v>8</v>
       </c>
       <c r="D35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F35" t="s">
         <v>16</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="3:7" x14ac:dyDescent="0.25">
@@ -1402,91 +1402,91 @@
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E36" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F36" t="s">
         <v>16</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F37" t="s">
         <v>16</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E38" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F38" t="s">
         <v>16</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E39" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F39" t="s">
         <v>16</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D40" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E40" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F40" t="s">
         <v>16</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E41" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F41" t="s">
         <v>16</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="42" spans="3:7" ht="30" x14ac:dyDescent="0.25">
       <c r="D42" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E42" t="s">
         <v>23</v>
@@ -1495,12 +1495,12 @@
         <v>16</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="43" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D43" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E43" t="s">
         <v>23</v>
@@ -1509,12 +1509,12 @@
         <v>16</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E44" t="s">
         <v>23</v>
@@ -1523,12 +1523,12 @@
         <v>16</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D45" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E45" t="s">
         <v>23</v>
@@ -1537,105 +1537,105 @@
         <v>16</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="3:7" ht="45" x14ac:dyDescent="0.25">
       <c r="D46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E46" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F46" t="s">
         <v>29</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="47" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D47" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E47" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F47" t="s">
         <v>29</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D48" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E48" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F48" t="s">
         <v>29</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D49" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E49" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F49" t="s">
         <v>29</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="50" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D50" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E50" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F50" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="51" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D51" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E51" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F51" t="s">
+        <v>105</v>
+      </c>
+      <c r="G51" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="52" spans="3:7" ht="45" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E52" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F52" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="53" spans="3:7" ht="30" x14ac:dyDescent="0.25">
@@ -1643,16 +1643,16 @@
         <v>8</v>
       </c>
       <c r="D53" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E53" t="s">
+        <v>115</v>
+      </c>
+      <c r="F53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G53" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F53" t="s">
-        <v>16</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="54" spans="3:7" x14ac:dyDescent="0.25">
@@ -1660,7 +1660,7 @@
         <v>8</v>
       </c>
       <c r="D54" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E54" t="s">
         <v>7</v>
@@ -1669,147 +1669,147 @@
         <v>16</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="55" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D55" t="s">
+        <v>118</v>
+      </c>
+      <c r="E55" t="s">
+        <v>78</v>
+      </c>
+      <c r="F55" t="s">
+        <v>29</v>
+      </c>
+      <c r="G55" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="E55" t="s">
-        <v>79</v>
-      </c>
-      <c r="F55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="56" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E56" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F56" t="s">
         <v>29</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="57" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D57" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E57" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F57" t="s">
         <v>29</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="58" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D58" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E58" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F58" t="s">
         <v>29</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="59" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D59" t="s">
+        <v>126</v>
+      </c>
+      <c r="E59" t="s">
+        <v>64</v>
+      </c>
+      <c r="F59" t="s">
+        <v>29</v>
+      </c>
+      <c r="G59" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="E59" t="s">
-        <v>65</v>
-      </c>
-      <c r="F59" t="s">
-        <v>29</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="60" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D60" t="s">
+        <v>128</v>
+      </c>
+      <c r="E60" t="s">
+        <v>64</v>
+      </c>
+      <c r="F60" t="s">
+        <v>29</v>
+      </c>
+      <c r="G60" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="E60" t="s">
-        <v>65</v>
-      </c>
-      <c r="F60" t="s">
-        <v>29</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="61" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D61" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E61" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F61" t="s">
         <v>29</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="62" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D62" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F62" t="s">
         <v>29</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="63" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D63" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E63" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F63" t="s">
         <v>29</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="64" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D64" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E64" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F64" t="s">
         <v>29</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="65" spans="3:7" x14ac:dyDescent="0.25">
@@ -1817,16 +1817,16 @@
         <v>8</v>
       </c>
       <c r="D65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E65" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F65" t="s">
         <v>29</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="66" spans="3:7" x14ac:dyDescent="0.25">
@@ -1855,7 +1855,7 @@
   <sheetData>
     <row r="3" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="3:7" x14ac:dyDescent="0.25">
@@ -1877,21 +1877,21 @@
     </row>
     <row r="8" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
         <v>143</v>
-      </c>
-      <c r="E8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="9" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
         <v>7</v>
@@ -1900,26 +1900,26 @@
         <v>16</v>
       </c>
       <c r="G9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" t="s">
         <v>43</v>
       </c>
-      <c r="E10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" t="s">
-        <v>44</v>
-      </c>
       <c r="G10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E11" t="s">
         <v>7</v>
@@ -1928,7 +1928,7 @@
         <v>16</v>
       </c>
       <c r="G11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="3:7" x14ac:dyDescent="0.25">
@@ -1942,7 +1942,7 @@
         <v>16</v>
       </c>
       <c r="G12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="3:7" x14ac:dyDescent="0.25">
@@ -1956,91 +1956,91 @@
         <v>16</v>
       </c>
       <c r="G13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14" t="s">
         <v>29</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F15" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="3:7" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F16" t="s">
         <v>29</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F17" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F18" t="s">
         <v>29</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>